<commit_message>
Merge Italy into the EU node across the four 2035 EMPIRE scenarios
The 2035 EMPIRE runs (GoRES, NECPEssentials, REPowerEU++, Trinity) were
re-solved with Italy folded into the EU aggregate, so every node-indexed
input and the installed-capacity / NTC / storage outputs the midterm SDDP
and the market chain read are regenerated.  No model code changes: the
zone mapping in empire_scenario.jl already routes any non-ES/FR/PT node
to EU.

Only the light, pipeline-relevant tables are committed here; the bulk
EMPIRE hourly scenario data (electricload/solar/wind/hydro), the
Stochastic_* input tabs and the operational result dumps are left out of
the commit.

config.toml: line_rating_factor 0.8 -> 1, redispatch power_flow DC -> AC,
from_saved = "BAL".
</commit_message>
<xml_diff>
--- a/Data/2035/GoRES/Input/Xlsx/Sets.xlsx
+++ b/Data/2035/GoRES/Input/Xlsx/Sets.xlsx
@@ -430,7 +430,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A52"/>
+  <dimension ref="A1:A51"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -785,13 +785,6 @@
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
-        <is>
-          <t>Italy</t>
-        </is>
-      </c>
-    </row>
-    <row r="52">
-      <c r="A52" t="inlineStr">
         <is>
           <t>Portugal</t>
         </is>
@@ -1412,7 +1405,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B105"/>
+  <dimension ref="A1:B103"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -2620,7 +2613,7 @@
     <row r="102">
       <c r="A102" t="inlineStr">
         <is>
-          <t>Italy</t>
+          <t>Portugal</t>
         </is>
       </c>
       <c r="B102" t="inlineStr">
@@ -2632,34 +2625,10 @@
     <row r="103">
       <c r="A103" t="inlineStr">
         <is>
-          <t>Italy</t>
+          <t>Portugal</t>
         </is>
       </c>
       <c r="B103" t="inlineStr">
-        <is>
-          <t>Li-Ion_BESS</t>
-        </is>
-      </c>
-    </row>
-    <row r="104">
-      <c r="A104" t="inlineStr">
-        <is>
-          <t>Portugal</t>
-        </is>
-      </c>
-      <c r="B104" t="inlineStr">
-        <is>
-          <t>Hydro Pump Storage</t>
-        </is>
-      </c>
-    </row>
-    <row r="105">
-      <c r="A105" t="inlineStr">
-        <is>
-          <t>Portugal</t>
-        </is>
-      </c>
-      <c r="B105" t="inlineStr">
         <is>
           <t>Li-Ion_BESS</t>
         </is>
@@ -2676,7 +2645,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B271"/>
+  <dimension ref="A1:B263"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -5576,12 +5545,12 @@
     <row r="243">
       <c r="A243" t="inlineStr">
         <is>
-          <t>EU</t>
+          <t>France</t>
         </is>
       </c>
       <c r="B243" t="inlineStr">
         <is>
-          <t>Italy</t>
+          <t>ES212</t>
         </is>
       </c>
     </row>
@@ -5593,7 +5562,7 @@
       </c>
       <c r="B244" t="inlineStr">
         <is>
-          <t>ES212</t>
+          <t>ES220</t>
         </is>
       </c>
     </row>
@@ -5605,7 +5574,7 @@
       </c>
       <c r="B245" t="inlineStr">
         <is>
-          <t>ES220</t>
+          <t>ES241</t>
         </is>
       </c>
     </row>
@@ -5617,7 +5586,7 @@
       </c>
       <c r="B246" t="inlineStr">
         <is>
-          <t>ES241</t>
+          <t>ES512</t>
         </is>
       </c>
     </row>
@@ -5629,7 +5598,7 @@
       </c>
       <c r="B247" t="inlineStr">
         <is>
-          <t>ES512</t>
+          <t>ES513</t>
         </is>
       </c>
     </row>
@@ -5641,55 +5610,55 @@
       </c>
       <c r="B248" t="inlineStr">
         <is>
-          <t>ES513</t>
+          <t>EU</t>
         </is>
       </c>
     </row>
     <row r="249">
       <c r="A249" t="inlineStr">
         <is>
-          <t>France</t>
+          <t>Portugal</t>
         </is>
       </c>
       <c r="B249" t="inlineStr">
         <is>
-          <t>EU</t>
+          <t>ES113</t>
         </is>
       </c>
     </row>
     <row r="250">
       <c r="A250" t="inlineStr">
         <is>
-          <t>France</t>
+          <t>Portugal</t>
         </is>
       </c>
       <c r="B250" t="inlineStr">
         <is>
-          <t>Italy</t>
+          <t>ES114</t>
         </is>
       </c>
     </row>
     <row r="251">
       <c r="A251" t="inlineStr">
         <is>
-          <t>Italy</t>
+          <t>Portugal</t>
         </is>
       </c>
       <c r="B251" t="inlineStr">
         <is>
-          <t>EU</t>
+          <t>ES415</t>
         </is>
       </c>
     </row>
     <row r="252">
       <c r="A252" t="inlineStr">
         <is>
-          <t>Italy</t>
+          <t>Portugal</t>
         </is>
       </c>
       <c r="B252" t="inlineStr">
         <is>
-          <t>France</t>
+          <t>ES419</t>
         </is>
       </c>
     </row>
@@ -5701,7 +5670,7 @@
       </c>
       <c r="B253" t="inlineStr">
         <is>
-          <t>ES113</t>
+          <t>ES431</t>
         </is>
       </c>
     </row>
@@ -5713,7 +5682,7 @@
       </c>
       <c r="B254" t="inlineStr">
         <is>
-          <t>ES114</t>
+          <t>ES432</t>
         </is>
       </c>
     </row>
@@ -5725,38 +5694,38 @@
       </c>
       <c r="B255" t="inlineStr">
         <is>
-          <t>ES415</t>
+          <t>ES615</t>
         </is>
       </c>
     </row>
     <row r="256">
       <c r="A256" t="inlineStr">
         <is>
-          <t>Portugal</t>
+          <t>ES113</t>
         </is>
       </c>
       <c r="B256" t="inlineStr">
         <is>
-          <t>ES419</t>
+          <t>ES111</t>
         </is>
       </c>
     </row>
     <row r="257">
       <c r="A257" t="inlineStr">
         <is>
-          <t>Portugal</t>
+          <t>ES111</t>
         </is>
       </c>
       <c r="B257" t="inlineStr">
         <is>
-          <t>ES431</t>
+          <t>ES113</t>
         </is>
       </c>
     </row>
     <row r="258">
       <c r="A258" t="inlineStr">
         <is>
-          <t>Portugal</t>
+          <t>ES422</t>
         </is>
       </c>
       <c r="B258" t="inlineStr">
@@ -5768,156 +5737,60 @@
     <row r="259">
       <c r="A259" t="inlineStr">
         <is>
-          <t>Portugal</t>
+          <t>ES432</t>
         </is>
       </c>
       <c r="B259" t="inlineStr">
         <is>
-          <t>ES615</t>
+          <t>ES422</t>
         </is>
       </c>
     </row>
     <row r="260">
       <c r="A260" t="inlineStr">
         <is>
-          <t>ES113</t>
+          <t>ES618</t>
         </is>
       </c>
       <c r="B260" t="inlineStr">
         <is>
-          <t>ES111</t>
+          <t>ES422</t>
         </is>
       </c>
     </row>
     <row r="261">
       <c r="A261" t="inlineStr">
         <is>
-          <t>ES111</t>
+          <t>ES422</t>
         </is>
       </c>
       <c r="B261" t="inlineStr">
         <is>
-          <t>ES113</t>
+          <t>ES618</t>
         </is>
       </c>
     </row>
     <row r="262">
       <c r="A262" t="inlineStr">
         <is>
-          <t>ES422</t>
+          <t>ES213</t>
         </is>
       </c>
       <c r="B262" t="inlineStr">
         <is>
-          <t>ES432</t>
+          <t>France</t>
         </is>
       </c>
     </row>
     <row r="263">
       <c r="A263" t="inlineStr">
         <is>
-          <t>ES432</t>
+          <t>France</t>
         </is>
       </c>
       <c r="B263" t="inlineStr">
         <is>
-          <t>ES422</t>
-        </is>
-      </c>
-    </row>
-    <row r="264">
-      <c r="A264" t="inlineStr">
-        <is>
-          <t>ES618</t>
-        </is>
-      </c>
-      <c r="B264" t="inlineStr">
-        <is>
-          <t>ES422</t>
-        </is>
-      </c>
-    </row>
-    <row r="265">
-      <c r="A265" t="inlineStr">
-        <is>
-          <t>ES422</t>
-        </is>
-      </c>
-      <c r="B265" t="inlineStr">
-        <is>
-          <t>ES618</t>
-        </is>
-      </c>
-    </row>
-    <row r="266">
-      <c r="A266" t="inlineStr">
-        <is>
           <t>ES213</t>
-        </is>
-      </c>
-      <c r="B266" t="inlineStr">
-        <is>
-          <t>France</t>
-        </is>
-      </c>
-    </row>
-    <row r="267">
-      <c r="A267" t="inlineStr">
-        <is>
-          <t>France</t>
-        </is>
-      </c>
-      <c r="B267" t="inlineStr">
-        <is>
-          <t>ES213</t>
-        </is>
-      </c>
-    </row>
-    <row r="268">
-      <c r="A268" t="inlineStr">
-        <is>
-          <t>ES511</t>
-        </is>
-      </c>
-      <c r="B268" t="inlineStr">
-        <is>
-          <t>Italy</t>
-        </is>
-      </c>
-    </row>
-    <row r="269">
-      <c r="A269" t="inlineStr">
-        <is>
-          <t>Italy</t>
-        </is>
-      </c>
-      <c r="B269" t="inlineStr">
-        <is>
-          <t>ES511</t>
-        </is>
-      </c>
-    </row>
-    <row r="270">
-      <c r="A270" t="inlineStr">
-        <is>
-          <t>ES523</t>
-        </is>
-      </c>
-      <c r="B270" t="inlineStr">
-        <is>
-          <t>Italy</t>
-        </is>
-      </c>
-    </row>
-    <row r="271">
-      <c r="A271" t="inlineStr">
-        <is>
-          <t>Italy</t>
-        </is>
-      </c>
-      <c r="B271" t="inlineStr">
-        <is>
-          <t>ES523</t>
         </is>
       </c>
     </row>
@@ -5932,7 +5805,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C271"/>
+  <dimension ref="A1:C263"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -10032,12 +9905,12 @@
     <row r="243">
       <c r="A243" t="inlineStr">
         <is>
-          <t>EU</t>
+          <t>France</t>
         </is>
       </c>
       <c r="B243" t="inlineStr">
         <is>
-          <t>Italy</t>
+          <t>ES212</t>
         </is>
       </c>
       <c r="C243" t="inlineStr">
@@ -10054,7 +9927,7 @@
       </c>
       <c r="B244" t="inlineStr">
         <is>
-          <t>ES212</t>
+          <t>ES220</t>
         </is>
       </c>
       <c r="C244" t="inlineStr">
@@ -10071,7 +9944,7 @@
       </c>
       <c r="B245" t="inlineStr">
         <is>
-          <t>ES220</t>
+          <t>ES241</t>
         </is>
       </c>
       <c r="C245" t="inlineStr">
@@ -10088,7 +9961,7 @@
       </c>
       <c r="B246" t="inlineStr">
         <is>
-          <t>ES241</t>
+          <t>ES512</t>
         </is>
       </c>
       <c r="C246" t="inlineStr">
@@ -10105,7 +9978,7 @@
       </c>
       <c r="B247" t="inlineStr">
         <is>
-          <t>ES512</t>
+          <t>ES513</t>
         </is>
       </c>
       <c r="C247" t="inlineStr">
@@ -10122,41 +9995,41 @@
       </c>
       <c r="B248" t="inlineStr">
         <is>
-          <t>ES513</t>
+          <t>EU</t>
         </is>
       </c>
       <c r="C248" t="inlineStr">
         <is>
-          <t>HVAC_OverheadLine</t>
+          <t>HVDC_Cable</t>
         </is>
       </c>
     </row>
     <row r="249">
       <c r="A249" t="inlineStr">
         <is>
-          <t>France</t>
+          <t>Portugal</t>
         </is>
       </c>
       <c r="B249" t="inlineStr">
         <is>
-          <t>EU</t>
+          <t>ES113</t>
         </is>
       </c>
       <c r="C249" t="inlineStr">
         <is>
-          <t>HVDC_Cable</t>
+          <t>HVAC_OverheadLine</t>
         </is>
       </c>
     </row>
     <row r="250">
       <c r="A250" t="inlineStr">
         <is>
-          <t>France</t>
+          <t>Portugal</t>
         </is>
       </c>
       <c r="B250" t="inlineStr">
         <is>
-          <t>Italy</t>
+          <t>ES114</t>
         </is>
       </c>
       <c r="C250" t="inlineStr">
@@ -10168,12 +10041,12 @@
     <row r="251">
       <c r="A251" t="inlineStr">
         <is>
-          <t>Italy</t>
+          <t>Portugal</t>
         </is>
       </c>
       <c r="B251" t="inlineStr">
         <is>
-          <t>EU</t>
+          <t>ES415</t>
         </is>
       </c>
       <c r="C251" t="inlineStr">
@@ -10185,12 +10058,12 @@
     <row r="252">
       <c r="A252" t="inlineStr">
         <is>
-          <t>Italy</t>
+          <t>Portugal</t>
         </is>
       </c>
       <c r="B252" t="inlineStr">
         <is>
-          <t>France</t>
+          <t>ES419</t>
         </is>
       </c>
       <c r="C252" t="inlineStr">
@@ -10207,7 +10080,7 @@
       </c>
       <c r="B253" t="inlineStr">
         <is>
-          <t>ES113</t>
+          <t>ES431</t>
         </is>
       </c>
       <c r="C253" t="inlineStr">
@@ -10224,7 +10097,7 @@
       </c>
       <c r="B254" t="inlineStr">
         <is>
-          <t>ES114</t>
+          <t>ES432</t>
         </is>
       </c>
       <c r="C254" t="inlineStr">
@@ -10241,7 +10114,7 @@
       </c>
       <c r="B255" t="inlineStr">
         <is>
-          <t>ES415</t>
+          <t>ES615</t>
         </is>
       </c>
       <c r="C255" t="inlineStr">
@@ -10253,12 +10126,12 @@
     <row r="256">
       <c r="A256" t="inlineStr">
         <is>
-          <t>Portugal</t>
+          <t>ES113</t>
         </is>
       </c>
       <c r="B256" t="inlineStr">
         <is>
-          <t>ES419</t>
+          <t>ES111</t>
         </is>
       </c>
       <c r="C256" t="inlineStr">
@@ -10270,12 +10143,12 @@
     <row r="257">
       <c r="A257" t="inlineStr">
         <is>
-          <t>Portugal</t>
+          <t>ES111</t>
         </is>
       </c>
       <c r="B257" t="inlineStr">
         <is>
-          <t>ES431</t>
+          <t>ES113</t>
         </is>
       </c>
       <c r="C257" t="inlineStr">
@@ -10287,7 +10160,7 @@
     <row r="258">
       <c r="A258" t="inlineStr">
         <is>
-          <t>Portugal</t>
+          <t>ES422</t>
         </is>
       </c>
       <c r="B258" t="inlineStr">
@@ -10304,12 +10177,12 @@
     <row r="259">
       <c r="A259" t="inlineStr">
         <is>
-          <t>Portugal</t>
+          <t>ES432</t>
         </is>
       </c>
       <c r="B259" t="inlineStr">
         <is>
-          <t>ES615</t>
+          <t>ES422</t>
         </is>
       </c>
       <c r="C259" t="inlineStr">
@@ -10321,12 +10194,12 @@
     <row r="260">
       <c r="A260" t="inlineStr">
         <is>
-          <t>ES113</t>
+          <t>ES618</t>
         </is>
       </c>
       <c r="B260" t="inlineStr">
         <is>
-          <t>ES111</t>
+          <t>ES422</t>
         </is>
       </c>
       <c r="C260" t="inlineStr">
@@ -10338,12 +10211,12 @@
     <row r="261">
       <c r="A261" t="inlineStr">
         <is>
-          <t>ES111</t>
+          <t>ES422</t>
         </is>
       </c>
       <c r="B261" t="inlineStr">
         <is>
-          <t>ES113</t>
+          <t>ES618</t>
         </is>
       </c>
       <c r="C261" t="inlineStr">
@@ -10355,168 +10228,32 @@
     <row r="262">
       <c r="A262" t="inlineStr">
         <is>
-          <t>ES422</t>
+          <t>ES213</t>
         </is>
       </c>
       <c r="B262" t="inlineStr">
         <is>
-          <t>ES432</t>
+          <t>France</t>
         </is>
       </c>
       <c r="C262" t="inlineStr">
         <is>
-          <t>HVAC_OverheadLine</t>
+          <t>HVDC_Cable</t>
         </is>
       </c>
     </row>
     <row r="263">
       <c r="A263" t="inlineStr">
         <is>
-          <t>ES432</t>
+          <t>France</t>
         </is>
       </c>
       <c r="B263" t="inlineStr">
         <is>
-          <t>ES422</t>
+          <t>ES213</t>
         </is>
       </c>
       <c r="C263" t="inlineStr">
-        <is>
-          <t>HVAC_OverheadLine</t>
-        </is>
-      </c>
-    </row>
-    <row r="264">
-      <c r="A264" t="inlineStr">
-        <is>
-          <t>ES618</t>
-        </is>
-      </c>
-      <c r="B264" t="inlineStr">
-        <is>
-          <t>ES422</t>
-        </is>
-      </c>
-      <c r="C264" t="inlineStr">
-        <is>
-          <t>HVAC_OverheadLine</t>
-        </is>
-      </c>
-    </row>
-    <row r="265">
-      <c r="A265" t="inlineStr">
-        <is>
-          <t>ES422</t>
-        </is>
-      </c>
-      <c r="B265" t="inlineStr">
-        <is>
-          <t>ES618</t>
-        </is>
-      </c>
-      <c r="C265" t="inlineStr">
-        <is>
-          <t>HVAC_OverheadLine</t>
-        </is>
-      </c>
-    </row>
-    <row r="266">
-      <c r="A266" t="inlineStr">
-        <is>
-          <t>ES213</t>
-        </is>
-      </c>
-      <c r="B266" t="inlineStr">
-        <is>
-          <t>France</t>
-        </is>
-      </c>
-      <c r="C266" t="inlineStr">
-        <is>
-          <t>HVDC_Cable</t>
-        </is>
-      </c>
-    </row>
-    <row r="267">
-      <c r="A267" t="inlineStr">
-        <is>
-          <t>France</t>
-        </is>
-      </c>
-      <c r="B267" t="inlineStr">
-        <is>
-          <t>ES213</t>
-        </is>
-      </c>
-      <c r="C267" t="inlineStr">
-        <is>
-          <t>HVDC_Cable</t>
-        </is>
-      </c>
-    </row>
-    <row r="268">
-      <c r="A268" t="inlineStr">
-        <is>
-          <t>ES511</t>
-        </is>
-      </c>
-      <c r="B268" t="inlineStr">
-        <is>
-          <t>Italy</t>
-        </is>
-      </c>
-      <c r="C268" t="inlineStr">
-        <is>
-          <t>HVDC_Cable</t>
-        </is>
-      </c>
-    </row>
-    <row r="269">
-      <c r="A269" t="inlineStr">
-        <is>
-          <t>Italy</t>
-        </is>
-      </c>
-      <c r="B269" t="inlineStr">
-        <is>
-          <t>ES511</t>
-        </is>
-      </c>
-      <c r="C269" t="inlineStr">
-        <is>
-          <t>HVDC_Cable</t>
-        </is>
-      </c>
-    </row>
-    <row r="270">
-      <c r="A270" t="inlineStr">
-        <is>
-          <t>ES523</t>
-        </is>
-      </c>
-      <c r="B270" t="inlineStr">
-        <is>
-          <t>Italy</t>
-        </is>
-      </c>
-      <c r="C270" t="inlineStr">
-        <is>
-          <t>HVDC_Cable</t>
-        </is>
-      </c>
-    </row>
-    <row r="271">
-      <c r="A271" t="inlineStr">
-        <is>
-          <t>Italy</t>
-        </is>
-      </c>
-      <c r="B271" t="inlineStr">
-        <is>
-          <t>ES523</t>
-        </is>
-      </c>
-      <c r="C271" t="inlineStr">
         <is>
           <t>HVDC_Cable</t>
         </is>
@@ -10533,7 +10270,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B540"/>
+  <dimension ref="A1:B525"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -16637,7 +16374,7 @@
     <row r="510">
       <c r="A510" t="inlineStr">
         <is>
-          <t>Italy</t>
+          <t>Portugal</t>
         </is>
       </c>
       <c r="B510" t="inlineStr">
@@ -16649,7 +16386,7 @@
     <row r="511">
       <c r="A511" t="inlineStr">
         <is>
-          <t>Italy</t>
+          <t>Portugal</t>
         </is>
       </c>
       <c r="B511" t="inlineStr">
@@ -16661,7 +16398,7 @@
     <row r="512">
       <c r="A512" t="inlineStr">
         <is>
-          <t>Italy</t>
+          <t>Portugal</t>
         </is>
       </c>
       <c r="B512" t="inlineStr">
@@ -16673,7 +16410,7 @@
     <row r="513">
       <c r="A513" t="inlineStr">
         <is>
-          <t>Italy</t>
+          <t>Portugal</t>
         </is>
       </c>
       <c r="B513" t="inlineStr">
@@ -16685,7 +16422,7 @@
     <row r="514">
       <c r="A514" t="inlineStr">
         <is>
-          <t>Italy</t>
+          <t>Portugal</t>
         </is>
       </c>
       <c r="B514" t="inlineStr">
@@ -16697,7 +16434,7 @@
     <row r="515">
       <c r="A515" t="inlineStr">
         <is>
-          <t>Italy</t>
+          <t>Portugal</t>
         </is>
       </c>
       <c r="B515" t="inlineStr">
@@ -16709,7 +16446,7 @@
     <row r="516">
       <c r="A516" t="inlineStr">
         <is>
-          <t>Italy</t>
+          <t>Portugal</t>
         </is>
       </c>
       <c r="B516" t="inlineStr">
@@ -16721,7 +16458,7 @@
     <row r="517">
       <c r="A517" t="inlineStr">
         <is>
-          <t>Italy</t>
+          <t>Portugal</t>
         </is>
       </c>
       <c r="B517" t="inlineStr">
@@ -16733,7 +16470,7 @@
     <row r="518">
       <c r="A518" t="inlineStr">
         <is>
-          <t>Italy</t>
+          <t>Portugal</t>
         </is>
       </c>
       <c r="B518" t="inlineStr">
@@ -16745,7 +16482,7 @@
     <row r="519">
       <c r="A519" t="inlineStr">
         <is>
-          <t>Italy</t>
+          <t>Portugal</t>
         </is>
       </c>
       <c r="B519" t="inlineStr">
@@ -16757,7 +16494,7 @@
     <row r="520">
       <c r="A520" t="inlineStr">
         <is>
-          <t>Italy</t>
+          <t>Portugal</t>
         </is>
       </c>
       <c r="B520" t="inlineStr">
@@ -16769,7 +16506,7 @@
     <row r="521">
       <c r="A521" t="inlineStr">
         <is>
-          <t>Italy</t>
+          <t>Portugal</t>
         </is>
       </c>
       <c r="B521" t="inlineStr">
@@ -16781,7 +16518,7 @@
     <row r="522">
       <c r="A522" t="inlineStr">
         <is>
-          <t>Italy</t>
+          <t>Portugal</t>
         </is>
       </c>
       <c r="B522" t="inlineStr">
@@ -16793,7 +16530,7 @@
     <row r="523">
       <c r="A523" t="inlineStr">
         <is>
-          <t>Italy</t>
+          <t>Portugal</t>
         </is>
       </c>
       <c r="B523" t="inlineStr">
@@ -16805,12 +16542,12 @@
     <row r="524">
       <c r="A524" t="inlineStr">
         <is>
-          <t>Italy</t>
+          <t>Portugal</t>
         </is>
       </c>
       <c r="B524" t="inlineStr">
         <is>
-          <t>Wind onshore</t>
+          <t>Wave</t>
         </is>
       </c>
     </row>
@@ -16821,186 +16558,6 @@
         </is>
       </c>
       <c r="B525" t="inlineStr">
-        <is>
-          <t>Bio</t>
-        </is>
-      </c>
-    </row>
-    <row r="526">
-      <c r="A526" t="inlineStr">
-        <is>
-          <t>Portugal</t>
-        </is>
-      </c>
-      <c r="B526" t="inlineStr">
-        <is>
-          <t>Bio CCS</t>
-        </is>
-      </c>
-    </row>
-    <row r="527">
-      <c r="A527" t="inlineStr">
-        <is>
-          <t>Portugal</t>
-        </is>
-      </c>
-      <c r="B527" t="inlineStr">
-        <is>
-          <t>Coal</t>
-        </is>
-      </c>
-    </row>
-    <row r="528">
-      <c r="A528" t="inlineStr">
-        <is>
-          <t>Portugal</t>
-        </is>
-      </c>
-      <c r="B528" t="inlineStr">
-        <is>
-          <t>Coal CCS</t>
-        </is>
-      </c>
-    </row>
-    <row r="529">
-      <c r="A529" t="inlineStr">
-        <is>
-          <t>Portugal</t>
-        </is>
-      </c>
-      <c r="B529" t="inlineStr">
-        <is>
-          <t>Gas CCGT</t>
-        </is>
-      </c>
-    </row>
-    <row r="530">
-      <c r="A530" t="inlineStr">
-        <is>
-          <t>Portugal</t>
-        </is>
-      </c>
-      <c r="B530" t="inlineStr">
-        <is>
-          <t>Gas CCS</t>
-        </is>
-      </c>
-    </row>
-    <row r="531">
-      <c r="A531" t="inlineStr">
-        <is>
-          <t>Portugal</t>
-        </is>
-      </c>
-      <c r="B531" t="inlineStr">
-        <is>
-          <t>Gas OCGT</t>
-        </is>
-      </c>
-    </row>
-    <row r="532">
-      <c r="A532" t="inlineStr">
-        <is>
-          <t>Portugal</t>
-        </is>
-      </c>
-      <c r="B532" t="inlineStr">
-        <is>
-          <t>Geo</t>
-        </is>
-      </c>
-    </row>
-    <row r="533">
-      <c r="A533" t="inlineStr">
-        <is>
-          <t>Portugal</t>
-        </is>
-      </c>
-      <c r="B533" t="inlineStr">
-        <is>
-          <t>Hydro regulated</t>
-        </is>
-      </c>
-    </row>
-    <row r="534">
-      <c r="A534" t="inlineStr">
-        <is>
-          <t>Portugal</t>
-        </is>
-      </c>
-      <c r="B534" t="inlineStr">
-        <is>
-          <t>Hydro run-of-the-river</t>
-        </is>
-      </c>
-    </row>
-    <row r="535">
-      <c r="A535" t="inlineStr">
-        <is>
-          <t>Portugal</t>
-        </is>
-      </c>
-      <c r="B535" t="inlineStr">
-        <is>
-          <t>Nuclear</t>
-        </is>
-      </c>
-    </row>
-    <row r="536">
-      <c r="A536" t="inlineStr">
-        <is>
-          <t>Portugal</t>
-        </is>
-      </c>
-      <c r="B536" t="inlineStr">
-        <is>
-          <t>Oil</t>
-        </is>
-      </c>
-    </row>
-    <row r="537">
-      <c r="A537" t="inlineStr">
-        <is>
-          <t>Portugal</t>
-        </is>
-      </c>
-      <c r="B537" t="inlineStr">
-        <is>
-          <t>Solar</t>
-        </is>
-      </c>
-    </row>
-    <row r="538">
-      <c r="A538" t="inlineStr">
-        <is>
-          <t>Portugal</t>
-        </is>
-      </c>
-      <c r="B538" t="inlineStr">
-        <is>
-          <t>Waste</t>
-        </is>
-      </c>
-    </row>
-    <row r="539">
-      <c r="A539" t="inlineStr">
-        <is>
-          <t>Portugal</t>
-        </is>
-      </c>
-      <c r="B539" t="inlineStr">
-        <is>
-          <t>Wave</t>
-        </is>
-      </c>
-    </row>
-    <row r="540">
-      <c r="A540" t="inlineStr">
-        <is>
-          <t>Portugal</t>
-        </is>
-      </c>
-      <c r="B540" t="inlineStr">
         <is>
           <t>Wind onshore</t>
         </is>
@@ -17017,7 +16574,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B137"/>
+  <dimension ref="A1:B133"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -18561,96 +18118,48 @@
     <row r="130">
       <c r="A130" t="inlineStr">
         <is>
-          <t>EU</t>
+          <t>ES113</t>
         </is>
       </c>
       <c r="B130" t="inlineStr">
         <is>
-          <t>Italy</t>
+          <t>ES111</t>
         </is>
       </c>
     </row>
     <row r="131">
       <c r="A131" t="inlineStr">
         <is>
-          <t>France</t>
+          <t>ES422</t>
         </is>
       </c>
       <c r="B131" t="inlineStr">
         <is>
-          <t>Italy</t>
+          <t>ES432</t>
         </is>
       </c>
     </row>
     <row r="132">
       <c r="A132" t="inlineStr">
         <is>
-          <t>ES113</t>
+          <t>ES618</t>
         </is>
       </c>
       <c r="B132" t="inlineStr">
         <is>
-          <t>ES111</t>
+          <t>ES422</t>
         </is>
       </c>
     </row>
     <row r="133">
       <c r="A133" t="inlineStr">
         <is>
-          <t>ES422</t>
+          <t>ES213</t>
         </is>
       </c>
       <c r="B133" t="inlineStr">
         <is>
-          <t>ES432</t>
-        </is>
-      </c>
-    </row>
-    <row r="134">
-      <c r="A134" t="inlineStr">
-        <is>
-          <t>ES618</t>
-        </is>
-      </c>
-      <c r="B134" t="inlineStr">
-        <is>
-          <t>ES422</t>
-        </is>
-      </c>
-    </row>
-    <row r="135">
-      <c r="A135" t="inlineStr">
-        <is>
-          <t>ES213</t>
-        </is>
-      </c>
-      <c r="B135" t="inlineStr">
-        <is>
           <t>France</t>
-        </is>
-      </c>
-    </row>
-    <row r="136">
-      <c r="A136" t="inlineStr">
-        <is>
-          <t>ES511</t>
-        </is>
-      </c>
-      <c r="B136" t="inlineStr">
-        <is>
-          <t>Italy</t>
-        </is>
-      </c>
-    </row>
-    <row r="137">
-      <c r="A137" t="inlineStr">
-        <is>
-          <t>ES523</t>
-        </is>
-      </c>
-      <c r="B137" t="inlineStr">
-        <is>
-          <t>Italy</t>
         </is>
       </c>
     </row>
@@ -18665,7 +18174,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C137"/>
+  <dimension ref="A1:C133"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -20844,12 +20353,12 @@
     <row r="130">
       <c r="A130" t="inlineStr">
         <is>
-          <t>EU</t>
+          <t>ES113</t>
         </is>
       </c>
       <c r="B130" t="inlineStr">
         <is>
-          <t>Italy</t>
+          <t>ES111</t>
         </is>
       </c>
       <c r="C130" t="inlineStr">
@@ -20861,12 +20370,12 @@
     <row r="131">
       <c r="A131" t="inlineStr">
         <is>
-          <t>France</t>
+          <t>ES422</t>
         </is>
       </c>
       <c r="B131" t="inlineStr">
         <is>
-          <t>Italy</t>
+          <t>ES432</t>
         </is>
       </c>
       <c r="C131" t="inlineStr">
@@ -20878,12 +20387,12 @@
     <row r="132">
       <c r="A132" t="inlineStr">
         <is>
-          <t>ES113</t>
+          <t>ES618</t>
         </is>
       </c>
       <c r="B132" t="inlineStr">
         <is>
-          <t>ES111</t>
+          <t>ES422</t>
         </is>
       </c>
       <c r="C132" t="inlineStr">
@@ -20895,83 +20404,15 @@
     <row r="133">
       <c r="A133" t="inlineStr">
         <is>
-          <t>ES422</t>
+          <t>ES213</t>
         </is>
       </c>
       <c r="B133" t="inlineStr">
         <is>
-          <t>ES432</t>
+          <t>France</t>
         </is>
       </c>
       <c r="C133" t="inlineStr">
-        <is>
-          <t>HVAC_OverheadLine</t>
-        </is>
-      </c>
-    </row>
-    <row r="134">
-      <c r="A134" t="inlineStr">
-        <is>
-          <t>ES618</t>
-        </is>
-      </c>
-      <c r="B134" t="inlineStr">
-        <is>
-          <t>ES422</t>
-        </is>
-      </c>
-      <c r="C134" t="inlineStr">
-        <is>
-          <t>HVAC_OverheadLine</t>
-        </is>
-      </c>
-    </row>
-    <row r="135">
-      <c r="A135" t="inlineStr">
-        <is>
-          <t>ES213</t>
-        </is>
-      </c>
-      <c r="B135" t="inlineStr">
-        <is>
-          <t>France</t>
-        </is>
-      </c>
-      <c r="C135" t="inlineStr">
-        <is>
-          <t>HVDC_Cable</t>
-        </is>
-      </c>
-    </row>
-    <row r="136">
-      <c r="A136" t="inlineStr">
-        <is>
-          <t>ES511</t>
-        </is>
-      </c>
-      <c r="B136" t="inlineStr">
-        <is>
-          <t>Italy</t>
-        </is>
-      </c>
-      <c r="C136" t="inlineStr">
-        <is>
-          <t>HVDC_Cable</t>
-        </is>
-      </c>
-    </row>
-    <row r="137">
-      <c r="A137" t="inlineStr">
-        <is>
-          <t>ES523</t>
-        </is>
-      </c>
-      <c r="B137" t="inlineStr">
-        <is>
-          <t>Italy</t>
-        </is>
-      </c>
-      <c r="C137" t="inlineStr">
         <is>
           <t>HVDC_Cable</t>
         </is>
@@ -20988,7 +20429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C54"/>
+  <dimension ref="A1:C53"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -21640,10 +21081,10 @@
         </is>
       </c>
       <c r="B51" t="n">
-        <v>52.946591</v>
+        <v>52.705838</v>
       </c>
       <c r="C51" t="n">
-        <v>10.934426</v>
+        <v>10.969925</v>
       </c>
     </row>
     <row r="52">
@@ -21662,26 +21103,13 @@
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>Italy</t>
+          <t>Portugal</t>
         </is>
       </c>
       <c r="B53" t="n">
-        <v>41.871941</v>
+        <v>39.399872</v>
       </c>
       <c r="C53" t="n">
-        <v>12.56738</v>
-      </c>
-    </row>
-    <row r="54">
-      <c r="A54" t="inlineStr">
-        <is>
-          <t>Portugal</t>
-        </is>
-      </c>
-      <c r="B54" t="n">
-        <v>39.399872</v>
-      </c>
-      <c r="C54" t="n">
         <v>-8.224454</v>
       </c>
     </row>

</xml_diff>